<commit_message>
Marca ARNALDO: nombre del torcedor, acuerdo de nombre/imagen y participación, brief creativo
- Sustituye FOLIO por ARNALDO en todo el dossier (FOLIO y LUMBRE quedan como reserva)
- Nuevo borrador de acuerdo con Arnaldo (licencia de nombre, firma e imagen; royalty/equity)
- Modelo financiero: parámetros de royalty y participación de Arnaldo
- Brief creativo para diseñador profesional e identidad provisional; v1/v2 archivadas
- Riesgos, decisiones, fuentes y plan de 180 días actualizados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CvqttADUwhWNoyN5jfGGtF
</commit_message>
<xml_diff>
--- a/PROYECTO_CIGARS_CUBA_2027/00_EXECUTIVE/Decision Matrix.xlsx
+++ b/PROYECTO_CIGARS_CUBA_2027/00_EXECUTIVE/Decision Matrix.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="172">
   <si>
     <t xml:space="preserve">Matriz de decisión — Estrategias (Proyecto C)</t>
   </si>
@@ -377,10 +377,10 @@
     <t xml:space="preserve">Nombre de marca definitivo</t>
   </si>
   <si>
-    <t xml:space="preserve">FOLIO / LUMBRE / VELADA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FOLIO, tras informe de registrabilidad</t>
+    <t xml:space="preserve">ARNALDO / FOLIO / LUMBRE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARNALDO (decidido por el promotor 10/10/2026), condicionado a consentimiento de Arnaldo e informe de registrabilidad</t>
   </si>
   <si>
     <t xml:space="preserve">Búsqueda EUIPO/OEPM/OCPI por agente</t>
@@ -407,6 +407,30 @@
     <t xml:space="preserve">D01–D03</t>
   </si>
   <si>
+    <t xml:space="preserve">D11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contraprestación de Arnaldo por nombre y colaboración</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A royalty 2% / B equity 10% con vesting / C mixta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B o C: equity con vesting alinea incentivos sin consumir caja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dictamen cubano sobre cobro legal; autorización del empleador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Promotor + abogados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fase 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D02, D10</t>
+  </si>
+  <si>
     <t xml:space="preserve">D10</t>
   </si>
   <si>
@@ -423,9 +447,6 @@
   </si>
   <si>
     <t xml:space="preserve">Abogado cubano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fase 0</t>
   </si>
   <si>
     <t xml:space="preserve">Condiciones verificables para avanzar (CONDITIONAL GO)</t>
@@ -1933,7 +1954,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -2239,6 +2260,32 @@
         <v>133</v>
       </c>
       <c r="H14" s="13" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="G15" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="H15" s="13" t="s">
         <v>80</v>
       </c>
     </row>
@@ -2269,12 +2316,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2282,24 +2329,24 @@
         <v>64</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="D5" s="6" t="n">
         <v>0</v>
@@ -2307,13 +2354,13 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="D6" s="6" t="n">
         <v>0</v>
@@ -2321,13 +2368,13 @@
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>0</v>
@@ -2335,13 +2382,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>0</v>
@@ -2349,13 +2396,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>0</v>
@@ -2363,13 +2410,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="D10" s="6" t="n">
         <v>0</v>
@@ -2377,13 +2424,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="D11" s="6" t="n">
         <v>0</v>
@@ -2391,13 +2438,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>0</v>
@@ -2405,7 +2452,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="4" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="D14" s="9" t="n">
         <f aca="false">SUM(D5:D12)</f>
@@ -2414,7 +2461,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="4" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="D15" s="14" t="str">
         <f aca="false">IF(D14=8,"GO a primer pedido piloto",IF(AND(D5=1,D6=1),"CONDITIONAL GO: continuar Fases 1–3","NO-GO a compromiso de capital: sólo Fase 0"))</f>

</xml_diff>

<commit_message>
Revisió des del punt de vista d'un inversor: coherència i transparència
- Dossier: noves pàgines d'economia unitària (imports exactes del model),
  escenaris («què ha de ser veritat») i Fase 0 / ús del primer euro (24 pàg.).
- Escenaris, business case i memo: coherència entre volum i demanda
  accessible (punts de venda necessaris), efecte de la remuneració del
  promotor, mida del negoci en euros i palanca d'origen alternatiu.
- C4 inclou un dictamen de sancions UE/EUA (via V1 a través de Habanos S.A.).
- Pla de 180 dies: el disseny professional passa després del Go (la Fase 0
  queda en 12.100 € a 90 dies, dins del sostre de 15.000 €).
- Noves decisions D12 (proposta a inversors) i D13 (origen alternatiu).
- Business Plan i brief d'identitat actualitzats a la Ruta A v2; rang de
  fonts S01–S51.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Cf1VjW9mqckGqcvuVgoNK
</commit_message>
<xml_diff>
--- a/PROYECTO_CIGARS_CUBA_2027/00_EXECUTIVE/Decision Matrix.xlsx
+++ b/PROYECTO_CIGARS_CUBA_2027/00_EXECUTIVE/Decision Matrix.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="186">
   <si>
     <t xml:space="preserve">Matriz de decisión — Estrategias (Proyecto C)</t>
   </si>
@@ -449,6 +449,48 @@
     <t xml:space="preserve">Abogado cubano</t>
   </si>
   <si>
+    <t xml:space="preserve">D12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Propuesta a inversores: importe, tramos e instrumento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sin inversores hasta el Go / tramos condicionados a C1–C8 / socio estratégico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tramos: Fase 0 con capital propio; capital externo sólo tras el Go y por hitos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resultado de la Fase 0; aportación del promotor; perfil de inversor buscado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Antes de presentar a inversores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D01, D09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Origen alternativo de ARNALDO (R. Dominicana / Nicaragua) si la vía cubana no se abre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sí / No / Sólo como plan B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plan B documentado: mejora el coste ≈2 €/u (arancel 0%), pero cambia el posicionamiento y el papel de Arnaldo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cotizaciones de fabricantes no cubanos; encaje legal de Arnaldo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comité Go/No-Go</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D01, D10</t>
+  </si>
+  <si>
     <t xml:space="preserve">Condiciones verificables para avanzar (CONDITIONAL GO)</t>
   </si>
   <si>
@@ -494,10 +536,10 @@
     <t xml:space="preserve">C4</t>
   </si>
   <si>
-    <t xml:space="preserve">Vía de pago verificada con banco español (y cubano) para el importe del primer pedido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carta/correo del banco</t>
+    <t xml:space="preserve">Vía de pago verificada con banco español (y cubano) para el importe del primer pedido y dictamen de sanciones UE/EE. UU. sobre la contraparte y el flujo de pagos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carta/correo del banco + dictamen de abogado de sanciones</t>
   </si>
   <si>
     <t xml:space="preserve">C5</t>
@@ -1954,7 +1996,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -2287,6 +2329,58 @@
       </c>
       <c r="H15" s="13" t="s">
         <v>80</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="G16" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="H16" s="13" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="s">
+        <v>148</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="G17" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="H17" s="13" t="s">
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -2316,12 +2410,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>142</v>
+        <v>156</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2329,24 +2423,24 @@
         <v>64</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>143</v>
+        <v>157</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>145</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>146</v>
+        <v>160</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>147</v>
+        <v>161</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="D5" s="6" t="n">
         <v>0</v>
@@ -2354,13 +2448,13 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="D6" s="6" t="n">
         <v>0</v>
@@ -2368,27 +2462,27 @@
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>154</v>
+        <v>168</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>0</v>
@@ -2396,13 +2490,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>158</v>
+        <v>172</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>159</v>
+        <v>173</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>0</v>
@@ -2410,13 +2504,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>162</v>
+        <v>176</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>163</v>
+        <v>177</v>
       </c>
       <c r="D10" s="6" t="n">
         <v>0</v>
@@ -2424,13 +2518,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>164</v>
+        <v>178</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="D11" s="6" t="n">
         <v>0</v>
@@ -2438,13 +2532,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>0</v>
@@ -2452,7 +2546,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="4" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
       <c r="D14" s="9" t="n">
         <f aca="false">SUM(D5:D12)</f>
@@ -2461,7 +2555,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="4" t="s">
-        <v>171</v>
+        <v>185</v>
       </c>
       <c r="D15" s="14" t="str">
         <f aca="false">IF(D14=8,"GO a primer pedido piloto",IF(AND(D5=1,D6=1),"CONDITIONAL GO: continuar Fases 1–3","NO-GO a compromiso de capital: sólo Fase 0"))</f>

</xml_diff>

<commit_message>
Rebranding: la marca passa a ARNALDO VALLÉS (nom i cognom del torcedor)
Oval de l'anella: ARNALDO VALLÉS en capitals en arc + signatura «Arnaldo
Vallés». Foto de referència retocada (original conservat), art vectorial,
maquetes, logotip, wordmark provisional i marca a foc regenerats. Tots els
documents, models i XLSX actualitzats; dossier reanomenat. Naming: DON VALLES
(EUA, puros, 2016) afegit com a anterioritat a analitzar (S62).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Cf1VjW9mqckGqcvuVgoNK
</commit_message>
<xml_diff>
--- a/PROYECTO_CIGARS_CUBA_2027/00_EXECUTIVE/Decision Matrix.xlsx
+++ b/PROYECTO_CIGARS_CUBA_2027/00_EXECUTIVE/Decision Matrix.xlsx
@@ -377,10 +377,10 @@
     <t xml:space="preserve">Nombre de marca definitivo</t>
   </si>
   <si>
-    <t xml:space="preserve">ARNALDO / FOLIO / LUMBRE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARNALDO (decidido por el promotor 10/10/2026), condicionado a consentimiento de Arnaldo e informe de registrabilidad</t>
+    <t xml:space="preserve">ARNALDO VALLÉS / FOLIO / LUMBRE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARNALDO VALLÉS (decidido por el promotor 17/10/2026; antes ARNALDO, 10/10/2026), condicionado a consentimiento de Arnaldo e informe de registrabilidad</t>
   </si>
   <si>
     <t xml:space="preserve">Búsqueda EUIPO/OEPM/OCPI por agente</t>
@@ -473,7 +473,7 @@
     <t xml:space="preserve">D13</t>
   </si>
   <si>
-    <t xml:space="preserve">Origen alternativo de ARNALDO (R. Dominicana / Nicaragua) si la vía cubana no se abre</t>
+    <t xml:space="preserve">Origen alternativo de ARNALDO VALLÉS (R. Dominicana / Nicaragua) si la vía cubana no se abre</t>
   </si>
   <si>
     <t xml:space="preserve">Sí / No / Sólo como plan B</t>
@@ -2227,7 +2227,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
         <v>115</v>
       </c>

</xml_diff>